<commit_message>
Initial work for Interim 3 (Q7). Fixed worked for previous questions (missing + gamma on theta_4 calculation)
</commit_message>
<xml_diff>
--- a/Interim2/Q6/ENME473_DrivingTorque.xlsx
+++ b/Interim2/Q6/ENME473_DrivingTorque.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="22" uniqueCount="11">
   <si>
     <t>Theta2_deg</t>
   </si>
@@ -95,7 +95,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="true"/>
-    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="2" max="2" width="12.42578125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -111,7 +111,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="0">
-        <v>3.3900611187725893</v>
+        <v>4.0866006541707272</v>
       </c>
     </row>
     <row r="3">
@@ -119,7 +119,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="0">
-        <v>6.5688072759441116</v>
+        <v>6.8036411504406082</v>
       </c>
     </row>
     <row r="4">
@@ -127,7 +127,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="0">
-        <v>7.6509170897069385</v>
+        <v>7.726131635099807</v>
       </c>
     </row>
     <row r="5">
@@ -135,7 +135,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="0">
-        <v>8.0841148737323252</v>
+        <v>8.09279916213438</v>
       </c>
     </row>
     <row r="6">
@@ -143,7 +143,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="0">
-        <v>8.2639045130638387</v>
+        <v>8.242389367979083</v>
       </c>
     </row>
     <row r="7">
@@ -151,7 +151,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="0">
-        <v>8.3297790371480929</v>
+        <v>8.2943733704872749</v>
       </c>
     </row>
     <row r="8">
@@ -159,7 +159,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="0">
-        <v>8.3393749358003806</v>
+        <v>8.2980761934999823</v>
       </c>
     </row>
     <row r="9">
@@ -167,7 +167,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="0">
-        <v>8.3191876649485668</v>
+        <v>8.2761402747838595</v>
       </c>
     </row>
     <row r="10">
@@ -175,7 +175,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="0">
-        <v>8.2823463234193504</v>
+        <v>8.2397627927151298</v>
       </c>
     </row>
     <row r="11">
@@ -183,7 +183,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="0">
-        <v>8.2357139293385693</v>
+        <v>8.1947814707245765</v>
       </c>
     </row>
     <row r="12">
@@ -191,7 +191,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="0">
-        <v>8.1830139617355311</v>
+        <v>8.144353003815473</v>
       </c>
     </row>
     <row r="13">
@@ -199,7 +199,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="0">
-        <v>8.1263146023215391</v>
+        <v>8.0902234635291261</v>
       </c>
     </row>
     <row r="14">
@@ -207,7 +207,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="0">
-        <v>8.0667764756213014</v>
+        <v>8.0333675370090791</v>
       </c>
     </row>
     <row r="15">
@@ -215,7 +215,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="0">
-        <v>8.0050477526293822</v>
+        <v>7.9743257746471246</v>
       </c>
     </row>
     <row r="16">
@@ -223,7 +223,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="0">
-        <v>7.9414811381082737</v>
+        <v>7.9133894479572113</v>
       </c>
     </row>
     <row r="17">
@@ -231,7 +231,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="0">
-        <v>7.8762568195049987</v>
+        <v>7.8507050497425803</v>
       </c>
     </row>
     <row r="18">
@@ -239,7 +239,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="0">
-        <v>7.8094538971834098</v>
+        <v>7.7863348362271338</v>
       </c>
     </row>
     <row r="19">
@@ -247,7 +247,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="0">
-        <v>7.741092700717874</v>
+        <v>7.7202925722862519</v>
       </c>
     </row>
     <row r="20">
@@ -255,7 +255,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="0">
-        <v>7.6711602184026484</v>
+        <v>7.6525649242830029</v>
       </c>
     </row>
     <row r="21">
@@ -263,7 +263,7 @@
         <v>19</v>
       </c>
       <c r="B21" s="0">
-        <v>7.5996255169174489</v>
+        <v>7.5831243664990273</v>
       </c>
     </row>
     <row r="22">
@@ -271,7 +271,7 @@
         <v>20</v>
       </c>
       <c r="B22" s="0">
-        <v>7.5264491206550766</v>
+        <v>7.5119369815012096</v>
       </c>
     </row>
     <row r="23">
@@ -279,7 +279,7 @@
         <v>21</v>
       </c>
       <c r="B23" s="0">
-        <v>7.4515886937902884</v>
+        <v>7.4389671459089843</v>
       </c>
     </row>
     <row r="24">
@@ -287,7 +287,7 @@
         <v>22</v>
       </c>
       <c r="B24" s="0">
-        <v>7.3750024349284704</v>
+        <v>7.3641802971622958</v>
       </c>
     </row>
     <row r="25">
@@ -295,7 +295,7 @@
         <v>23</v>
       </c>
       <c r="B25" s="0">
-        <v>7.2966510465950067</v>
+        <v>7.2875445106376073</v>
       </c>
     </row>
     <row r="26">
@@ -303,7 +303,7 @@
         <v>24</v>
       </c>
       <c r="B26" s="0">
-        <v>7.2164988141692481</v>
+        <v>7.2090313379589297</v>
       </c>
     </row>
     <row r="27">
@@ -311,7 +311,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="0">
-        <v>7.1345141294061714</v>
+        <v>7.1286161881550951</v>
       </c>
     </row>
     <row r="28">
@@ -319,7 +319,7 @@
         <v>26</v>
       </c>
       <c r="B28" s="0">
-        <v>7.0506696704310317</v>
+        <v>7.0462784289999538</v>
       </c>
     </row>
     <row r="29">
@@ -327,7 +327,7 @@
         <v>27</v>
       </c>
       <c r="B29" s="0">
-        <v>6.9649423729342246</v>
+        <v>6.962001320743398</v>
       </c>
     </row>
     <row r="30">
@@ -335,7 +335,7 @@
         <v>28</v>
       </c>
       <c r="B30" s="0">
-        <v>6.8773132784583275</v>
+        <v>6.8757718533435446</v>
       </c>
     </row>
     <row r="31">
@@ -343,7 +343,7 @@
         <v>29</v>
       </c>
       <c r="B31" s="0">
-        <v>6.7877673144805</v>
+        <v>6.7875805321549301</v>
       </c>
     </row>
     <row r="32">
@@ -351,7 +351,7 @@
         <v>30</v>
       </c>
       <c r="B32" s="0">
-        <v>6.696293040932245</v>
+        <v>6.6974211402716826</v>
       </c>
     </row>
     <row r="33">
@@ -359,7 +359,7 @@
         <v>31</v>
       </c>
       <c r="B33" s="0">
-        <v>6.60288238483062</v>
+        <v>6.6052904949447635</v>
       </c>
     </row>
     <row r="34">
@@ -367,7 +367,7 @@
         <v>32</v>
       </c>
       <c r="B34" s="0">
-        <v>6.5075303762890533</v>
+        <v>6.5111882085455122</v>
       </c>
     </row>
     <row r="35">
@@ -375,7 +375,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="0">
-        <v>6.410234893728445</v>
+        <v>6.4151164600760557</v>
       </c>
     </row>
     <row r="36">
@@ -383,7 +383,7 @@
         <v>34</v>
       </c>
       <c r="B36" s="0">
-        <v>6.3109964225891755</v>
+        <v>6.3170797803637484</v>
       </c>
     </row>
     <row r="37">
@@ -391,7 +391,7 @@
         <v>35</v>
       </c>
       <c r="B37" s="0">
-        <v>6.2098178295888928</v>
+        <v>6.2170848522621407</v>
       </c>
     </row>
     <row r="38">
@@ -399,7 +399,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="0">
-        <v>6.1067041531438875</v>
+        <v>6.1151403260505175</v>
       </c>
     </row>
     <row r="39">
@@ -407,7 +407,7 @@
         <v>37</v>
       </c>
       <c r="B39" s="0">
-        <v>6.0016624096907769</v>
+        <v>6.0112566495412905</v>
       </c>
     </row>
     <row r="40">
@@ -415,7 +415,7 @@
         <v>38</v>
       </c>
       <c r="B40" s="0">
-        <v>5.8947014151204238</v>
+        <v>5.9054459120118681</v>
       </c>
     </row>
     <row r="41">
@@ -423,7 +423,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="0">
-        <v>5.7858316202446485</v>
+        <v>5.7977217008725495</v>
       </c>
     </row>
     <row r="42">
@@ -431,7 +431,7 @@
         <v>40</v>
       </c>
       <c r="B42" s="0">
-        <v>5.675064959075069</v>
+        <v>5.6880989698967861</v>
       </c>
     </row>
     <row r="43">
@@ -439,7 +439,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="0">
-        <v>5.5624147086472409</v>
+        <v>5.5765939178288191</v>
       </c>
     </row>
     <row r="44">
@@ -447,7 +447,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="0">
-        <v>5.4478953591361572</v>
+        <v>5.4632238762172829</v>
       </c>
     </row>
     <row r="45">
@@ -455,7 +455,7 @@
         <v>43</v>
       </c>
       <c r="B45" s="0">
-        <v>5.3315224930564771</v>
+        <v>5.3480072053823591</v>
       </c>
     </row>
     <row r="46">
@@ -463,7 +463,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="0">
-        <v>5.2133126724068717</v>
+        <v>5.2309631974953952</v>
       </c>
     </row>
     <row r="47">
@@ -471,7 +471,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="0">
-        <v>5.093283332692276</v>
+        <v>5.1121119858256137</v>
       </c>
     </row>
     <row r="48">
@@ -479,7 +479,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="0">
-        <v>4.9714526828338919</v>
+        <v>4.9914744592839515</v>
       </c>
     </row>
     <row r="49">
@@ -487,7 +487,7 @@
         <v>47</v>
       </c>
       <c r="B49" s="0">
-        <v>4.8478396100501833</v>
+        <v>4.8690721814650679</v>
       </c>
     </row>
     <row r="50">
@@ -495,7 +495,7 @@
         <v>48</v>
       </c>
       <c r="B50" s="0">
-        <v>4.7224635888607853</v>
+        <v>4.7449273134547978</v>
       </c>
     </row>
     <row r="51">
@@ -503,7 +503,7 @@
         <v>49</v>
       </c>
       <c r="B51" s="0">
-        <v>4.5953445934269821</v>
+        <v>4.6190625397290246</v>
       </c>
     </row>
     <row r="52">
@@ -511,7 +511,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="0">
-        <v>4.4665030124976823</v>
+        <v>4.4915009965230732</v>
       </c>
     </row>
     <row r="53">
@@ -519,7 +519,7 @@
         <v>51</v>
       </c>
       <c r="B53" s="0">
-        <v>4.3359595662768422</v>
+        <v>4.3622662020955332</v>
       </c>
     </row>
     <row r="54">
@@ -527,7 +527,7 @@
         <v>52</v>
       </c>
       <c r="B54" s="0">
-        <v>4.2037352245684865</v>
+        <v>4.2313819883497219</v>
       </c>
     </row>
     <row r="55">
@@ -535,7 +535,7 @@
         <v>53</v>
       </c>
       <c r="B55" s="0">
-        <v>4.0698511255881558</v>
+        <v>4.0988724333078226</v>
       </c>
     </row>
     <row r="56">
@@ -543,7 +543,7 @@
         <v>54</v>
       </c>
       <c r="B56" s="0">
-        <v>3.9343284948551438</v>
+        <v>3.9647617939591799</v>
       </c>
     </row>
     <row r="57">
@@ -551,7 +551,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="0">
-        <v>3.7971885635988114</v>
+        <v>3.8290744390241684</v>
       </c>
     </row>
     <row r="58">
@@ -559,7 +559,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="0">
-        <v>3.6584524861245553</v>
+        <v>3.6918347811898586</v>
       </c>
     </row>
     <row r="59">
@@ -567,7 +567,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="0">
-        <v>3.518141255591055</v>
+        <v>3.5530672083830979</v>
       </c>
     </row>
     <row r="60">
@@ -575,7 +575,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="0">
-        <v>3.3762756176502333</v>
+        <v>3.4127960136506563</v>
       </c>
     </row>
     <row r="61">
@@ -583,7 +583,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="0">
-        <v>3.2328759813953356</v>
+        <v>3.2710453232159025</v>
       </c>
     </row>
     <row r="62">
@@ -591,7 +591,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="0">
-        <v>3.0879623270505356</v>
+        <v>3.1278390222754773</v>
       </c>
     </row>
     <row r="63">
@@ -599,7 +599,7 @@
         <v>61</v>
       </c>
       <c r="B63" s="0">
-        <v>2.9415541098176616</v>
+        <v>2.9832006780897866</v>
       </c>
     </row>
     <row r="64">
@@ -607,7 +607,7 @@
         <v>62</v>
       </c>
       <c r="B64" s="0">
-        <v>2.7936701592718802</v>
+        <v>2.8371534599059225</v>
       </c>
     </row>
     <row r="65">
@@ -615,7 +615,7 @@
         <v>63</v>
       </c>
       <c r="B65" s="0">
-        <v>2.6443285736688464</v>
+        <v>2.689720055232157</v>
       </c>
     </row>
     <row r="66">
@@ -623,7 +623,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="0">
-        <v>2.49354660849</v>
+        <v>2.5409225819586601</v>
       </c>
     </row>
     <row r="67">
@@ -631,7 +631,7 @@
         <v>65</v>
       </c>
       <c r="B67" s="0">
-        <v>2.3413405585115741</v>
+        <v>2.3907824957898467</v>
       </c>
     </row>
     <row r="68">
@@ -639,7 +639,7 @@
         <v>66</v>
       </c>
       <c r="B68" s="0">
-        <v>2.1877256326349701</v>
+        <v>2.2393204924192465</v>
       </c>
     </row>
     <row r="69">
@@ -647,7 +647,7 @@
         <v>67</v>
       </c>
       <c r="B69" s="0">
-        <v>2.0327158206625184</v>
+        <v>2.0865564038380331</v>
       </c>
     </row>
     <row r="70">
@@ -655,7 +655,7 @@
         <v>68</v>
       </c>
       <c r="B70" s="0">
-        <v>1.8763237511430275</v>
+        <v>1.9325090881236688</v>
       </c>
     </row>
     <row r="71">
@@ -663,7 +663,7 @@
         <v>69</v>
       </c>
       <c r="B71" s="0">
-        <v>1.7185605393454893</v>
+        <v>1.777196312004063</v>
       </c>
     </row>
     <row r="72">
@@ -671,7 +671,7 @@
         <v>70</v>
       </c>
       <c r="B72" s="0">
-        <v>1.5594356243480096</v>
+        <v>1.62063462543652</v>
       </c>
     </row>
     <row r="73">
@@ -679,7 +679,7 @@
         <v>71</v>
       </c>
       <c r="B73" s="0">
-        <v>1.3989565941528044</v>
+        <v>1.462839227378661</v>
       </c>
     </row>
     <row r="74">
@@ -687,7 +687,7 @@
         <v>72</v>
       </c>
       <c r="B74" s="0">
-        <v>1.2371289976571551</v>
+        <v>1.3038238218602789</v>
       </c>
     </row>
     <row r="75">
@@ -695,7 +695,7 @@
         <v>73</v>
       </c>
       <c r="B75" s="0">
-        <v>1.0739561422276647</v>
+        <v>1.1436004633919294</v>
       </c>
     </row>
     <row r="76">
@@ -703,7 +703,7 @@
         <v>74</v>
       </c>
       <c r="B76" s="0">
-        <v>0.9094388755413777</v>
+        <v>0.98217939066691062</v>
       </c>
     </row>
     <row r="77">
@@ -711,7 +711,7 @@
         <v>75</v>
       </c>
       <c r="B77" s="0">
-        <v>0.74357535027730859</v>
+        <v>0.81956884743028224</v>
       </c>
     </row>
     <row r="78">
@@ -719,7 +719,7 @@
         <v>76</v>
       </c>
       <c r="B78" s="0">
-        <v>0.57636077016942511</v>
+        <v>0.65577488930209382</v>
       </c>
     </row>
     <row r="79">
@@ -727,7 +727,7 @@
         <v>77</v>
       </c>
       <c r="B79" s="0">
-        <v>0.40778711587449534</v>
+        <v>0.49080117525412126</v>
       </c>
     </row>
     <row r="80">
@@ -735,7 +735,7 @@
         <v>78</v>
       </c>
       <c r="B80" s="0">
-        <v>0.23784284907509695</v>
+        <v>0.32464874235344632</v>
       </c>
     </row>
     <row r="81">
@@ -743,7 +743,7 @@
         <v>79</v>
       </c>
       <c r="B81" s="0">
-        <v>0.066512593242420218</v>
+        <v>0.15731576230550959</v>
       </c>
     </row>
     <row r="82">
@@ -751,7 +751,7 @@
         <v>80</v>
       </c>
       <c r="B82" s="0">
-        <v>-0.10622321045443628</v>
+        <v>-0.011202721738772042</v>
       </c>
     </row>
     <row r="83">
@@ -759,7 +759,7 @@
         <v>81</v>
       </c>
       <c r="B83" s="0">
-        <v>-0.28038867346228824</v>
+        <v>-0.18091507969566245</v>
       </c>
     </row>
     <row r="84">
@@ -767,7 +767,7 @@
         <v>82</v>
       </c>
       <c r="B84" s="0">
-        <v>-0.45601285748616172</v>
+        <v>-0.35183340197991253</v>
       </c>
     </row>
     <row r="85">
@@ -775,7 +775,7 @@
         <v>83</v>
       </c>
       <c r="B85" s="0">
-        <v>-0.63313020013257848</v>
+        <v>-0.52397383141942733</v>
       </c>
     </row>
     <row r="86">
@@ -783,7 +783,7 @@
         <v>84</v>
       </c>
       <c r="B86" s="0">
-        <v>-0.81178096855360316</v>
+        <v>-0.69735692111013226</v>
       </c>
     </row>
     <row r="87">
@@ -791,7 +791,7 @@
         <v>85</v>
       </c>
       <c r="B87" s="0">
-        <v>-0.99201174008266391</v>
+        <v>-0.87200801945397488</v>
       </c>
     </row>
     <row r="88">
@@ -799,7 +799,7 @@
         <v>86</v>
       </c>
       <c r="B88" s="0">
-        <v>-1.173875907372667</v>
+        <v>-1.0479576832560773</v>
       </c>
     </row>
     <row r="89">
@@ -807,7 +807,7 @@
         <v>87</v>
       </c>
       <c r="B89" s="0">
-        <v>-1.3574342034072979</v>
+        <v>-1.2252421191748113</v>
       </c>
     </row>
     <row r="90">
@@ -815,7 +815,7 @@
         <v>88</v>
       </c>
       <c r="B90" s="0">
-        <v>-1.542755238692374</v>
+        <v>-1.4039036529305151</v>
       </c>
     </row>
     <row r="91">
@@ -823,7 +823,7 @@
         <v>89</v>
       </c>
       <c r="B91" s="0">
-        <v>-1.7299160385748595</v>
+        <v>-1.5839912243617931</v>
       </c>
     </row>
     <row r="92">
@@ -831,7 +831,7 @@
         <v>90</v>
       </c>
       <c r="B92" s="0">
-        <v>-1.9190025624579703</v>
+        <v>-1.765560904499824</v>
       </c>
     </row>
     <row r="93">
@@ -839,7 +839,7 @@
         <v>91</v>
       </c>
       <c r="B93" s="0">
-        <v>-2.1101101779332225</v>
+        <v>-1.9486764280665563</v>
       </c>
     </row>
     <row r="94">
@@ -847,7 +847,7 @@
         <v>92</v>
       </c>
       <c r="B94" s="0">
-        <v>-2.3033440504691405</v>
+        <v>-2.1334097308515614</v>
       </c>
     </row>
     <row r="95">
@@ -855,7 +855,7 @@
         <v>93</v>
       </c>
       <c r="B95" s="0">
-        <v>-2.4988193917422028</v>
+        <v>-2.3198414757995551</v>
       </c>
     </row>
     <row r="96">
@@ -863,7 +863,7 @@
         <v>94</v>
       </c>
       <c r="B96" s="0">
-        <v>-2.6966614847410404</v>
+        <v>-2.5080615436575595</v>
       </c>
     </row>
     <row r="97">
@@ -871,7 +871,7 @@
         <v>95</v>
       </c>
       <c r="B97" s="0">
-        <v>-2.8970053681607788</v>
+        <v>-2.6981694527033997</v>
       </c>
     </row>
     <row r="98">
@@ -879,7 +879,7 @@
         <v>96</v>
       </c>
       <c r="B98" s="0">
-        <v>-3.0999950115273163</v>
+        <v>-2.8902746559865502</v>
       </c>
     </row>
     <row r="99">
@@ -887,7 +887,7 @@
         <v>97</v>
       </c>
       <c r="B99" s="0">
-        <v>-3.30578173879988</v>
+        <v>-3.0844966416024322</v>
       </c>
     </row>
     <row r="100">
@@ -895,7 +895,7 @@
         <v>98</v>
       </c>
       <c r="B100" s="0">
-        <v>-3.5145215511446657</v>
+        <v>-3.2809647287855812</v>
       </c>
     </row>
     <row r="101">
@@ -903,7 +903,7 @@
         <v>99</v>
       </c>
       <c r="B101" s="0">
-        <v>-3.7263708428055806</v>
+        <v>-3.4798174056170113</v>
       </c>
     </row>
     <row r="102">
@@ -911,7 +911,7 @@
         <v>100</v>
       </c>
       <c r="B102" s="0">
-        <v>-3.9414797723727797</v>
+        <v>-3.6812009863029083</v>
       </c>
     </row>
     <row r="103">
@@ -919,7 +919,7 @@
         <v>101</v>
       </c>
       <c r="B103" s="0">
-        <v>-4.1599822060642726</v>
+        <v>-3.8852672673952453</v>
       </c>
     </row>
     <row r="104">
@@ -927,7 +927,7 @@
         <v>102</v>
       </c>
       <c r="B104" s="0">
-        <v>-4.3819806279238929</v>
+        <v>-4.0921697179423537</v>
       </c>
     </row>
     <row r="105">
@@ -935,7 +935,7 @@
         <v>103</v>
       </c>
       <c r="B105" s="0">
-        <v>-4.6075236146301784</v>
+        <v>-4.3020575252577231</v>
       </c>
     </row>
     <row r="106">
@@ -943,7 +943,7 @@
         <v>104</v>
       </c>
       <c r="B106" s="0">
-        <v>-4.8365722375520903</v>
+        <v>-4.5150664997766938</v>
       </c>
     </row>
     <row r="107">
@@ -951,7 +951,7 @@
         <v>105</v>
       </c>
       <c r="B107" s="0">
-        <v>-5.0689498119289604</v>
+        <v>-4.7313053625054442</v>
       </c>
     </row>
     <row r="108">
@@ -959,7 +959,7 @@
         <v>106</v>
       </c>
       <c r="B108" s="0">
-        <v>-5.304266305042642</v>
+        <v>-4.9508352057867366</v>
       </c>
     </row>
     <row r="109">
@@ -967,7 +967,7 @@
         <v>107</v>
       </c>
       <c r="B109" s="0">
-        <v>-5.5418036490414249</v>
+        <v>-5.17363878415002</v>
       </c>
     </row>
     <row r="110">
@@ -975,7 +975,7 @@
         <v>108</v>
       </c>
       <c r="B110" s="0">
-        <v>-5.7803397719718985</v>
+        <v>-5.3995745108272741</v>
       </c>
     </row>
     <row r="111">
@@ -983,7 +983,7 @@
         <v>109</v>
       </c>
       <c r="B111" s="0">
-        <v>-6.0178747960532926</v>
+        <v>-5.628307190928564</v>
       </c>
     </row>
     <row r="112">
@@ -991,7 +991,7 @@
         <v>110</v>
       </c>
       <c r="B112" s="0">
-        <v>-6.2511977353202051</v>
+        <v>-5.8592028950902906</v>
       </c>
     </row>
     <row r="113">
@@ -999,7 +999,7 @@
         <v>111</v>
       </c>
       <c r="B113" s="0">
-        <v>-6.4751867987851295</v>
+        <v>-6.0911676949711646</v>
       </c>
     </row>
     <row r="114">
@@ -1007,7 +1007,7 @@
         <v>112</v>
       </c>
       <c r="B114" s="0">
-        <v>-6.6816522176102664</v>
+        <v>-6.3223969324313218</v>
       </c>
     </row>
     <row r="115">
@@ -1015,7 +1015,7 @@
         <v>113</v>
       </c>
       <c r="B115" s="0">
-        <v>-6.85736774251688</v>
+        <v>-6.5499789539911024</v>
       </c>
     </row>
     <row r="116">
@@ -1023,7 +1023,7 @@
         <v>114</v>
       </c>
       <c r="B116" s="0">
-        <v>-6.9806082109642516</v>
+        <v>-6.7692564580695009</v>
       </c>
     </row>
     <row r="117">
@@ -1031,7 +1031,7 @@
         <v>115</v>
       </c>
       <c r="B117" s="0">
-        <v>-7.0148120897058952</v>
+        <v>-6.9727730357899276</v>
       </c>
     </row>
     <row r="118">
@@ -1039,7 +1039,7 @@
         <v>116</v>
       </c>
       <c r="B118" s="0">
-        <v>-6.8964125854840672</v>
+        <v>-7.1484871782140802</v>
       </c>
     </row>
     <row r="119">
@@ -1047,7 +1047,7 @@
         <v>117</v>
       </c>
       <c r="B119" s="0">
-        <v>-6.510065865569624</v>
+        <v>-7.276644435213246</v>
       </c>
     </row>
     <row r="120">
@@ -1055,7 +1055,7 @@
         <v>118</v>
       </c>
       <c r="B120" s="0">
-        <v>-5.634429505906791</v>
+        <v>-7.3240836038609221</v>
       </c>
     </row>
     <row r="121">
@@ -1063,7 +1063,7 @@
         <v>119</v>
       </c>
       <c r="B121" s="0">
-        <v>-3.8120010315634687</v>
+        <v>-7.2333789711248215</v>
       </c>
     </row>
     <row r="122">
@@ -1071,7 +1071,7 @@
         <v>120</v>
       </c>
       <c r="B122" s="0">
-        <v>0.0036959332916062238</v>
+        <v>-6.900930627653115</v>
       </c>
     </row>
     <row r="124">
@@ -1121,7 +1121,7 @@
         <v>7</v>
       </c>
       <c r="B130" s="0">
-        <v>8.3393749358003806</v>
+        <v>8.2980761934999823</v>
       </c>
     </row>
     <row r="131">
@@ -1137,7 +1137,7 @@
         <v>9</v>
       </c>
       <c r="B132" s="0">
-        <v>-7.0148120897058952</v>
+        <v>-7.3240836038609221</v>
       </c>
     </row>
     <row r="133">
@@ -1145,7 +1145,7 @@
         <v>10</v>
       </c>
       <c r="B133" s="0">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>